<commit_message>
Daily EOD data and reports for 2026-07-30
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260730.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260730.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.33</v>
+        <v>1.315</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>-0.025</v>
+        <v>-0.04</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>-1.85%</t>
+          <t>-2.95%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>203730.73</v>
+        <v>201433.01</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>-3829.52</v>
+        <v>-6127.24</v>
       </c>
     </row>
     <row r="5">
@@ -515,24 +515,24 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2.16</v>
+        <v>2.15</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>-0.03</v>
+        <v>-0.04</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>-1.37%</t>
+          <t>-1.83%</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>151200</v>
+        <v>150500</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>-2100</v>
+        <v>-2800</v>
       </c>
     </row>
     <row r="6">
@@ -542,24 +542,24 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>0.93</v>
+        <v>0.945</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>-0.055</v>
+        <v>-0.04</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>-5.58%</t>
+          <t>-4.06%</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
         <v>57458</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>53435.94</v>
+        <v>54297.81</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>-3160.19</v>
+        <v>-2298.32</v>
       </c>
     </row>
     <row r="7">
@@ -569,24 +569,24 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>59.36</v>
+        <v>59.15</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>-0.82</v>
+        <v>-1.03</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>-1.36%</t>
+          <t>-1.71%</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
         <v>11065</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>656818.4</v>
+        <v>654494.75</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>-9073.299999999999</v>
+        <v>-11396.95</v>
       </c>
     </row>
     <row r="8">
@@ -623,14 +623,14 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>178.36</v>
+        <v>178.25</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>-0.3</v>
+        <v>-0.41</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-0.17%</t>
+          <t>-0.23%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
@@ -650,24 +650,24 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>0.735</v>
+        <v>0.73</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>-0.025</v>
+        <v>-0.03</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>-3.29%</t>
+          <t>-3.95%</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
         <v>10000</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>7350</v>
+        <v>7300</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>-250</v>
+        <v>-300</v>
       </c>
     </row>
     <row r="11">
@@ -677,24 +677,24 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>126.92</v>
+        <v>127.93</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>-1.15</v>
+        <v>-0.14</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-0.90%</t>
+          <t>-0.11%</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>507680</v>
+        <v>511720</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-4600</v>
+        <v>-560</v>
       </c>
     </row>
     <row r="12">
@@ -704,24 +704,24 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>0.25</v>
+        <v>0.245</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0</v>
+        <v>-0.005</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>-2.00%</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
         <v>20000</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>5000</v>
+        <v>4900</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>0</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="13">
@@ -758,24 +758,24 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>0.08</v>
+        <v>0.081</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>-0.001</v>
+        <v>0</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>-1.23%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E14" s="3" t="n">
         <v>9412</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>752.96</v>
+        <v>762.37</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>-9.41</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -785,24 +785,24 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>0</v>
+        <v>0.11</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>-0.105</v>
+        <v>0.005</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>4.76%</t>
         </is>
       </c>
       <c r="E15" s="3" t="n">
         <v>6000</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>0</v>
+        <v>660</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>-630</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>38.32</v>
+        <v>38.15</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>0.38</v>
+        <v>0.21</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1.00%</t>
+          <t>0.55%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>32.825</v>
+        <v>32.9</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.16</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0.26%</t>
+          <t>0.49%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>42278.6</v>
+        <v>42375.2</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>109.48</v>
+        <v>206.08</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1628378.9</v>
+        <v>1628575.42</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>-24942.95</v>
+        <v>-24746.43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>